<commit_message>
deleted a rouge exe file hiding in crime/cri_agr/ that was 80MB big! It was a random VPN, I don't know why or how it was there, but I did a threat assessment and concluded I accidently downloaded it during my research aggregation. It is gone. Also updates some research notes fora couple pathways, still many many more to go
</commit_message>
<xml_diff>
--- a/data/Influence Matrix.xlsx
+++ b/data/Influence Matrix.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/0396cb379e3a3ab8/Documents/Projects/Society_v1/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/0396cb379e3a3ab8/Documents/Projects/Society_v1/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="411" documentId="8_{ED65F0B3-21E7-4477-B09D-7F37D962E108}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8A211A96-FA66-436B-8368-067F38B88D1B}"/>
   <bookViews>
-    <workbookView xWindow="1920" yWindow="1680" windowWidth="20370" windowHeight="10980" xr2:uid="{D7722B4C-434F-4E8B-BF65-156EC5BBE20D}"/>
+    <workbookView xWindow="28680" yWindow="1755" windowWidth="20640" windowHeight="11040" xr2:uid="{D7722B4C-434F-4E8B-BF65-156EC5BBE20D}"/>
   </bookViews>
   <sheets>
     <sheet name="Influence Matrix" sheetId="1" r:id="rId1"/>
@@ -10016,6 +10016,30 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
+  <conditionalFormatting sqref="B2 C3 D4 E5 F6 G7 H8 I9 J10 K11 L12 M13 N14 O15 P16 Q17 R18 S19 T20 U21 V22 W23 X24 Y25 Z26 AA27 AB28 AC29 AD30 AE31 AF32 AG33 AH34 AI35 AJ36 AK37 AN40 AO41 AP42 AQ43">
+    <cfRule type="colorScale" priority="6">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FF5A8AC6"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B2 L12 AQ43 M13 C3 D4 E5 F6 G7 H8 I9 J10 K11 N14 O15 P16 Q17 R18 S19 T20 U21 V22 W23 X24 Y25 Z26 AA27 AB28 AC29 AD30 AE31 AF32 AG33 AH34 AI35 AJ36 AK37 AN40 AO41 AP42">
+    <cfRule type="colorScale" priority="42">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
   <conditionalFormatting sqref="B2">
     <cfRule type="colorScale" priority="9">
       <colorScale>
@@ -10025,6 +10049,18 @@
         <color rgb="FFF8696B"/>
         <color rgb="FFFCFCFF"/>
         <color rgb="FF5A8AC6"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B45 L55 AQ86 M56 C46 D47 E48 F49 G50 H51 I52 J53 K54 N57 O58 P59 Q60 R61 S62 T63 U64 V65 W66 X67 Y68 Z69 AA70 AB71 AC72 AD73 AE74 AF75 AG76 AH77 AI78 AJ79 AK80 AL81 AM82 AN83 AO84 AP85">
+    <cfRule type="colorScale" priority="30">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
       </colorScale>
     </cfRule>
   </conditionalFormatting>
@@ -10052,19 +10088,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C3 B2 D4 E5 F6 G7 H8 I9 J10 K11 L12 M13 N14 O15 P16 Q17 R18 S19 T20 U21 V22 W23 X24 Y25 Z26 AA27 AB28 AC29 AD30 AE31 AF32 AG33 AH34 AI35 AJ36 AK37 AN40 AO41 AP42 AQ43">
-    <cfRule type="colorScale" priority="6">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFCFCFF"/>
-        <color rgb="FF5A8AC6"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="E5 D4 F6 G7 H8 I9 J10 X24 AH34 AI35">
+  <conditionalFormatting sqref="D4 E5 F6 G7 H8 I9 J10 X24 AH34 AI35">
     <cfRule type="colorScale" priority="11">
       <colorScale>
         <cfvo type="min"/>
@@ -10088,31 +10112,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="L12 B2 AQ43 M13 C3 D4 E5 F6 G7 H8 I9 J10 K11 N14 O15 P16 Q17 R18 S19 T20 U21 V22 W23 X24 Y25 Z26 AA27 AB28 AC29 AD30 AE31 AF32 AG33 AH34 AI35 AJ36 AK37 AN40 AO41 AP42">
-    <cfRule type="colorScale" priority="42">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="L55 B45 AQ86 M56 C46 D47 E48 F49 G50 H51 I52 J53 K54 N57 O58 P59 Q60 R61 S62 T63 U64 V65 W66 X67 Y68 Z69 AA70 AB71 AC72 AD73 AE74 AF75 AG76 AH77 AI78 AJ79 AK80 AL81 AM82 AN83 AO84 AP85">
-    <cfRule type="colorScale" priority="30">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="AL38 AM39">
+  <conditionalFormatting sqref="AM39 AL38">
     <cfRule type="colorScale" priority="1">
       <colorScale>
         <cfvo type="min"/>

</xml_diff>

<commit_message>
AV1 Anatomy of the 42 now at version v3.1.
</commit_message>
<xml_diff>
--- a/data/Influence Matrix.xlsx
+++ b/data/Influence Matrix.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/0396cb379e3a3ab8/Documents/Projects/Society_v1/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="411" documentId="8_{ED65F0B3-21E7-4477-B09D-7F37D962E108}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8A211A96-FA66-436B-8368-067F38B88D1B}"/>
+  <xr:revisionPtr revIDLastSave="423" documentId="8_{ED65F0B3-21E7-4477-B09D-7F37D962E108}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{BA47FF1C-0053-4C7D-A614-AE4B7C266E48}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="1755" windowWidth="20640" windowHeight="11040" xr2:uid="{D7722B4C-434F-4E8B-BF65-156EC5BBE20D}"/>
   </bookViews>
@@ -2711,7 +2711,7 @@
         <v>Cost of Living</v>
       </c>
       <c r="B7" s="24">
-        <v>0.19</v>
+        <v>0.15</v>
       </c>
       <c r="C7" s="23">
         <v>-0.16</v>
@@ -9861,7 +9861,7 @@
     </customSheetView>
   </customSheetViews>
   <conditionalFormatting sqref="A2:XFD2">
-    <cfRule type="colorScale" priority="10">
+    <cfRule type="colorScale" priority="12">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -9873,7 +9873,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A2:XFD37 A40:XFD43">
-    <cfRule type="colorScale" priority="8">
+    <cfRule type="colorScale" priority="10">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -9885,7 +9885,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A4:XFD4">
-    <cfRule type="colorScale" priority="12">
+    <cfRule type="colorScale" priority="14">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -9897,7 +9897,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A6:XFD6">
-    <cfRule type="colorScale" priority="13">
+    <cfRule type="colorScale" priority="15">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -9909,7 +9909,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A7:XFD7">
-    <cfRule type="colorScale" priority="14">
+    <cfRule type="colorScale" priority="16">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -9921,7 +9921,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A8:XFD8">
-    <cfRule type="colorScale" priority="15">
+    <cfRule type="colorScale" priority="17">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -9933,7 +9933,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A9:XFD9">
-    <cfRule type="colorScale" priority="16">
+    <cfRule type="colorScale" priority="18">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -9945,7 +9945,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A10:XFD10">
-    <cfRule type="colorScale" priority="17">
+    <cfRule type="colorScale" priority="19">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -9957,7 +9957,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A24:XFD24 M26">
-    <cfRule type="colorScale" priority="18">
+    <cfRule type="colorScale" priority="20">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -9969,7 +9969,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A34:XFD34">
-    <cfRule type="colorScale" priority="22">
+    <cfRule type="colorScale" priority="24">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -9981,7 +9981,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A35:XFD35">
-    <cfRule type="colorScale" priority="19">
+    <cfRule type="colorScale" priority="21">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -9993,7 +9993,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A38:XFD38">
-    <cfRule type="colorScale" priority="4">
+    <cfRule type="colorScale" priority="6">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -10005,31 +10005,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A39:XFD39">
-    <cfRule type="colorScale" priority="3">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B2 C3 D4 E5 F6 G7 H8 I9 J10 K11 L12 M13 N14 O15 P16 Q17 R18 S19 T20 U21 V22 W23 X24 Y25 Z26 AA27 AB28 AC29 AD30 AE31 AF32 AG33 AH34 AI35 AJ36 AK37 AN40 AO41 AP42 AQ43">
-    <cfRule type="colorScale" priority="6">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFCFCFF"/>
-        <color rgb="FF5A8AC6"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B2 L12 AQ43 M13 C3 D4 E5 F6 G7 H8 I9 J10 K11 N14 O15 P16 Q17 R18 S19 T20 U21 V22 W23 X24 Y25 Z26 AA27 AB28 AC29 AD30 AE31 AF32 AG33 AH34 AI35 AJ36 AK37 AN40 AO41 AP42">
-    <cfRule type="colorScale" priority="42">
+    <cfRule type="colorScale" priority="5">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -10041,7 +10017,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B2">
-    <cfRule type="colorScale" priority="9">
+    <cfRule type="colorScale" priority="11">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -10052,20 +10028,8 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B45 L55 AQ86 M56 C46 D47 E48 F49 G50 H51 I52 J53 K54 N57 O58 P59 Q60 R61 S62 T63 U64 V65 W66 X67 Y68 Z69 AA70 AB71 AC72 AD73 AE74 AF75 AG76 AH77 AI78 AJ79 AK80 AL81 AM82 AN83 AO84 AP85">
-    <cfRule type="colorScale" priority="30">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
   <conditionalFormatting sqref="B43:AP43 AQ42 B42:AO42 AP41:AQ41 B41:AN41 AO40:AQ40 B40:AM40 AL37:AQ37 B37:AJ37 AK36:AQ36 B36:AI36 AJ35:AQ35 B35:AH35 AI34:AQ34 B34:AG34 AH33:AQ33 B33:AF33 AG32:AQ32 B32:AE32 AF31:AQ31 B31:AD31 AE30:AQ30 B30:AC30 AD29:AQ29 B29:AB29 AC28:AQ28 B28:AA28 AB27:AQ27 B27:Z27 AA26:AQ26 Z25:AQ25 B25:X25 Y24:AQ24 B24:W24 X23:AQ23 B23:V23 W22:AQ22 B22:U22 V21:AQ21 B21:T21 U20:AQ20 B20:S20 T19:AQ19 B19:R19 S18:AQ18 B18:Q18 R17:AQ17 B17:P17 Q16:AQ16 B16:O16 P15:AQ15 B15:N15 O14:AQ14 B14:M14 N13:AQ13 B13:L13 M12:AQ12 B12:K12 L11:AQ11 B11:J11 K10:AQ10 B10:I10 J9:AQ9 B9:H9 I8:AQ8 B8:G8 H7:AQ7 B7:F7 G6:AQ6 B6:E6 F5:AQ5 B5:D5 E4:AQ4 B4:C4 D3:AQ3 B3 C2:AQ2 B26:Y26">
-    <cfRule type="colorScale" priority="23">
+    <cfRule type="colorScale" priority="25">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -10077,7 +10041,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B2:AQ37 B40:AQ43">
-    <cfRule type="colorScale" priority="25">
+    <cfRule type="colorScale" priority="27">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -10088,8 +10052,20 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="D4 E5 F6 G7 H8 I9 J10 X24 AH34 AI35">
-    <cfRule type="colorScale" priority="11">
+  <conditionalFormatting sqref="C3 B2 D4 E5 F6 G7 H8 I9 J10 K11 L12 M13 N14 O15 P16 Q17 R18 S19 T20 U21 V22 W23 X24 Y25 Z26 AA27 AB28 AC29 AD30 AE31 AF32 AG33 AH34 AI35 AJ36 AK37 AN40 AO41 AP42 AQ43">
+    <cfRule type="colorScale" priority="8">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FF5A8AC6"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E5 D4 F6 G7 H8 I9 J10 X24 AH34 AI35">
+    <cfRule type="colorScale" priority="13">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -10101,7 +10077,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="I8:XFD8 A8:G8 G6:XFD6 A6:E6 E4:XFD4 A4:C4 C2:XFD2 A2 J9:XFD9 A9:H9 K10:XFD10 A10:I10 N13:XFD13 A13:L13 W22:XFD22 A22:U22 Y24:XFD24 A24:W24 AI34:XFD34 A34:AG34 AJ35:XFD35 A35:AH35">
-    <cfRule type="colorScale" priority="5">
+    <cfRule type="colorScale" priority="7">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -10112,8 +10088,32 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="AM39 AL38">
-    <cfRule type="colorScale" priority="1">
+  <conditionalFormatting sqref="L12 B2 AQ43 M13 C3 D4 E5 F6 G7 H8 I9 J10 K11 N14 O15 P16 Q17 R18 S19 T20 U21 V22 W23 X24 Y25 Z26 AA27 AB28 AC29 AD30 AE31 AF32 AG33 AH34 AI35 AJ36 AK37 AN40 AO41 AP42">
+    <cfRule type="colorScale" priority="44">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="L55 B45 AQ86 M56 C46 D47 E48 F49 G50 H51 I52 J53 K54 N57 O58 P59 Q60 R61 S62 T63 U64 V65 W66 X67 Y68 Z69 AA70 AB71 AC72 AD73 AE74 AF75 AG76 AH77 AI78 AJ79 AK80 AL81 AM82 AN83 AO84 AP85">
+    <cfRule type="colorScale" priority="32">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="AL38 AM39">
+    <cfRule type="colorScale" priority="3">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -10125,7 +10125,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AO40:AP40 AP41 O14:AK14 K10 J9:K9 I8:K8 F5 D3:E3 B3 C2:E2 H9 H10:I10 O16 O17:P17 O18:Q18 O19:R19 T21 T22:U22 T23:V23 T24:W24 Z27 Z28:AA28 Z29:AB29 Z30:AC30 Z31:AD31 Z32:AE32 Z33:AF33 Z34:AG34 Z35:AH35 Z36:AI36 Z37:AJ37 Z40:AM40 Z41:AN41 Z42:AO42 Z43:AP43 G8:G12 T25:X25 O20:S25 F2:L3 E4:F4 AQ14:AQ32 H7:K7 L7:L11 G4:L6 AM24:AP28 P15:AK15 Q16:AK16 R17:AK17 S18:AK18 T19:AK19 U20:AK20 V21:AK21 W22:AK22 X23:AK23 Y24:AL24 Z25:AL25 AA26:AL26 AB27:AL27 AC28:AL28 AD29:AP29 AE30:AP30 AF31:AP31 AG32:AP32 AQ34:AQ37 AH33:AQ33 AI34:AP34 AJ35:AP35 AK36:AP36 AL37:AP37 AQ40:AQ42 N13:AK13 M2:AQ12 AN13:AQ13 AN14:AP23 AL13:AM23 M15:N25 M14 H11:J11 H12:K12 H35:Y37 L24:L25 H24:K34 G24:G37 G13:L23 F7:F16 D6:E16 D17:F37 D5 B4:C37 L26:Y34 B40:Y43">
-    <cfRule type="colorScale" priority="212">
+    <cfRule type="colorScale" priority="214">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -10137,7 +10137,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AO83:AP83 AP84 AN82:AP82 O57:AK57 M55 K53 J52:K52 I51:K51 B49:E49 F48 B48:D48 B47:C47 D46:E46 B46 C45:E45 H52 H53:I53 H54:J54 H55:K55 H56:L56 O60:P60 O61:Q61 O62:R62 T64 T65:U65 T66:V66 T67:W67 Z70 Z71:AA71 Z72:AB72 Z73:AC73 Z74:AD74 Z75:AE75 Z76:AF76 Z77:AG77 Z78:AH78 Z79:AI79 Z80:AJ80 Z81:AK81 Z82:AL82 Z83:AM83 Z84:AN84 Z85:AO85 Z86:AP86 G51:G86 H59:J86 K59:O59 K71:Y86 T68:X68 O63:S68 N58 H57:M58 B50:F86 F45:M46 E47:F47 AQ57:AQ75 H50:K50 L50:M54 G47:M49 AM68:AP71 P58:AK58 Q59:AK59 R60:AK60 S61:AK61 T62:AK62 U63:AK63 V64:AK64 W65:AK65 X66:AK66 Y67:AK67 Z68:AL68 AA69:AL69 AB70:AL70 AC71:AL71 AD72:AP72 AE73:AP73 AF74:AP74 AG75:AP75 AQ77:AQ80 AH76:AQ76 AI77:AP77 AJ78:AP78 AK79:AP79 AL80:AP80 AQ82:AQ85 AM81:AQ81 N45:AQ56 AL57:AP67 O69:Y70 K60:N70">
-    <cfRule type="colorScale" priority="27">
+    <cfRule type="colorScale" priority="29">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -10149,7 +10149,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AP42 AQ43 AO41 AN40 AK37 AJ36 AI35 AH34 AG33 AF32 AE31 AD30 AC29 AB28 AA27 Z26 Y25 X24 W23 V22 U21 T20 S19 R18 Q17 P16 O15 N14 M13 L12 K11 J10 I9 H8 G7 F6 E5 D4 C3 B2">
-    <cfRule type="colorScale" priority="40">
+    <cfRule type="colorScale" priority="42">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -10159,7 +10159,7 @@
         <color rgb="FF5A8AC6"/>
       </colorScale>
     </cfRule>
-    <cfRule type="colorScale" priority="41">
+    <cfRule type="colorScale" priority="43">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -10171,7 +10171,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AP85 AQ86 AO84 AN83 AM82 AL81 AK80 AJ79 AI78 AH77 AG76 AF75 AE74 AD73 AC72 AB71 AA70 Z69 Y68 X67 W66 V65 U64 T63 S62 R61 Q60 P59 O58 N57 M56 L55 K54 J53 I52 H51 G50 F49 E48 D47 C46 B45">
-    <cfRule type="colorScale" priority="28">
+    <cfRule type="colorScale" priority="30">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -10181,7 +10181,7 @@
         <color rgb="FF5A8AC6"/>
       </colorScale>
     </cfRule>
-    <cfRule type="colorScale" priority="29">
+    <cfRule type="colorScale" priority="31">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -10193,7 +10193,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AR43:XFD43 A43:AP43 AQ42:XFD42 A42:AO42 AP41:XFD41 A41:AN41 AO40:XFD40 A40:AM40 AL37:XFD37 A37:AJ37 AK36:XFD36 A36:AI36 AJ35:XFD35 A35:AH35 AI34:XFD34 A34:AG34 AH33:XFD33 A33:AF33 AG32:XFD32 A32:AE32 AF31:XFD31 A31:AD31 AE30:XFD30 A30:AC30 AD29:XFD29 A29:AB29 AC28:XFD28 A28:AA28 AB27:XFD27 A27:Z27 AA26:XFD26 Z25:XFD25 A25:X25 Y24:XFD24 A24:W24 X23:XFD23 A23:V23 W22:XFD22 A22:U22 V21:XFD21 A21:T21 U20:XFD20 A20:S20 T19:XFD19 A19:R19 S18:XFD18 A18:Q18 R17:XFD17 A17:P17 Q16:XFD16 A16:O16 P15:XFD15 A15:N15 O14:XFD14 A14:M14 N13:XFD13 A13:L13 M12:XFD12 A12:K12 L11:XFD11 A11:J11 K10:XFD10 A10:I10 J9:XFD9 A9:H9 I8:XFD8 A8:G8 H7:XFD7 A7:F7 G6:XFD6 A6:E6 F5:XFD5 A5:D5 E4:XFD4 A4:C4 D3:XFD3 A3:B3 C2:XFD2 A2 A26:Y26">
-    <cfRule type="colorScale" priority="7">
+    <cfRule type="colorScale" priority="9">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -10201,6 +10201,18 @@
         <color rgb="FFF8696B"/>
         <color rgb="FFFFEB84"/>
         <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B7:AQ7">
+    <cfRule type="colorScale" priority="1">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
       </colorScale>
     </cfRule>
   </conditionalFormatting>
@@ -10360,7 +10372,7 @@
       </c>
       <c r="D6" s="35">
         <f>'Influence Matrix'!B7</f>
-        <v>0.19</v>
+        <v>0.15</v>
       </c>
       <c r="G6" t="s">
         <v>78</v>

</xml_diff>